<commit_message>
Finalizing SPICE, EXCEL, WORD docs
</commit_message>
<xml_diff>
--- a/EXCEL FILEOVI/ZAVRSNI EXCEL - PRORACUN.xlsx
+++ b/EXCEL FILEOVI/ZAVRSNI EXCEL - PRORACUN.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/523341e057c2d1b5/Documents/2526 - LJETNI SEMESTAR/Bachelor-Thesis/EXCEL FILEOVI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="685" documentId="8_{2396A90B-B910-459B-ACE8-58213C55B081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE3DAAEC-E9AB-482A-B2F2-ACDE84DC2332}"/>
+  <xr:revisionPtr revIDLastSave="874" documentId="8_{2396A90B-B910-459B-ACE8-58213C55B081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F448193F-E5E0-4E0C-9637-52AD7A5DA0F3}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{B4FD3550-17E7-4D46-90CC-DFB7D5127C87}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="3" xr2:uid="{B4FD3550-17E7-4D46-90CC-DFB7D5127C87}"/>
   </bookViews>
   <sheets>
     <sheet name="SZE" sheetId="1" r:id="rId1"/>
     <sheet name="SZC" sheetId="2" r:id="rId2"/>
+    <sheet name="B" sheetId="4" r:id="rId3"/>
+    <sheet name="AB" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="43">
   <si>
     <t>Ucc</t>
   </si>
@@ -51,10 +53,40 @@
     <t>Uul</t>
   </si>
   <si>
-    <t>Ibq</t>
+    <t>Umt</t>
   </si>
   <si>
     <t>Rbb</t>
+  </si>
+  <si>
+    <t>Rc</t>
+  </si>
+  <si>
+    <t>hfe</t>
+  </si>
+  <si>
+    <t>Rt = 550 ohm</t>
+  </si>
+  <si>
+    <t>Rt = 1100 ohm</t>
+  </si>
+  <si>
+    <t>Rt = 2200 ohm</t>
+  </si>
+  <si>
+    <t>Rt = 3300 ohm</t>
+  </si>
+  <si>
+    <t>Rt = 4400 ohm</t>
+  </si>
+  <si>
+    <t>Re</t>
+  </si>
+  <si>
+    <t>Rt</t>
+  </si>
+  <si>
+    <t>Ibq</t>
   </si>
   <si>
     <t>Icq</t>
@@ -63,52 +95,40 @@
     <t>Uceq</t>
   </si>
   <si>
-    <t>hfe</t>
+    <t>Rac</t>
+  </si>
+  <si>
+    <t>hie</t>
   </si>
   <si>
     <t>Av</t>
   </si>
   <si>
-    <t>Rac</t>
+    <t>Uceq,m,pp</t>
   </si>
   <si>
-    <t>Re</t>
+    <t>Uceq,M,pp</t>
   </si>
   <si>
-    <t>Rt</t>
+    <t>Uiz,M,pp</t>
   </si>
   <si>
-    <t>Rc</t>
+    <t>Uiz, M, pp</t>
   </si>
   <si>
-    <t>hie</t>
+    <t>Uiz</t>
   </si>
   <si>
-    <t>Umt</t>
-  </si>
-  <si>
-    <t>Rt = 2200 ohm</t>
-  </si>
-  <si>
-    <t>Rt = 550 ohm</t>
-  </si>
-  <si>
-    <t>Rt = 1100 ohm</t>
-  </si>
-  <si>
-    <t>Rt = 3300 ohm</t>
-  </si>
-  <si>
-    <t>Rt = 4400 ohm</t>
-  </si>
-  <si>
-    <t>η [%]</t>
+    <t>Uiz [V]</t>
   </si>
   <si>
     <t>Pcc [W]</t>
   </si>
   <si>
     <t>Pout [W]</t>
+  </si>
+  <si>
+    <t>η [%]</t>
   </si>
   <si>
     <t>theta 1</t>
@@ -144,34 +164,26 @@
     <t>THD [%]</t>
   </si>
   <si>
-    <t>Uceq,m,pp</t>
+    <t>Ube</t>
   </si>
   <si>
-    <t>Uiz</t>
+    <t>Pt [W]</t>
   </si>
   <si>
-    <t>Uceq,M,pp</t>
-  </si>
-  <si>
-    <t>Uiz,M,pp</t>
-  </si>
-  <si>
-    <t>Uiz, M, pp</t>
-  </si>
-  <si>
-    <t>Uiz [V]</t>
+    <t>stupanj djelovanja %</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.000E+00"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.000000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -194,12 +206,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -240,7 +258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -250,7 +268,11 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -268,10 +290,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -592,24 +610,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25837755-7B05-4086-B92B-A6987546BB78}">
   <dimension ref="A1:AH45"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="14.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="13" width="12.06640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.59765625" bestFit="1" customWidth="1"/>
-    <col min="16" max="20" width="12.06640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="12.06640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="14.86328125" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="12.06640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="30" max="34" width="12.06640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="20" width="12" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="12" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="12" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="34" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:34">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -617,7 +635,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:34">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -625,7 +643,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:34">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -633,15 +651,15 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:34">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:34">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -649,67 +667,67 @@
         <v>820000</v>
       </c>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:34">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2">
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:34">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2">
         <v>380</v>
       </c>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A12" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="H12" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="O12" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
-      <c r="V12" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
-      <c r="AA12" s="9"/>
-      <c r="AC12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="AD12" s="9"/>
-      <c r="AE12" s="9"/>
-      <c r="AF12" s="9"/>
-      <c r="AG12" s="9"/>
-      <c r="AH12" s="9"/>
-    </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:34">
+      <c r="A12" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="H12" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="O12" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="13"/>
+      <c r="S12" s="13"/>
+      <c r="T12" s="13"/>
+      <c r="V12" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="W12" s="13"/>
+      <c r="X12" s="13"/>
+      <c r="Y12" s="13"/>
+      <c r="Z12" s="13"/>
+      <c r="AA12" s="13"/>
+      <c r="AC12" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD12" s="13"/>
+      <c r="AE12" s="13"/>
+      <c r="AF12" s="13"/>
+      <c r="AG12" s="13"/>
+      <c r="AH12" s="13"/>
+    </row>
+    <row r="13" spans="1:34">
       <c r="A13" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B13" s="4">
         <v>250</v>
@@ -727,7 +745,7 @@
         <v>3000</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="4">
         <v>250</v>
@@ -745,7 +763,7 @@
         <v>3000</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="P13" s="4">
         <v>250</v>
@@ -763,7 +781,7 @@
         <v>3000</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="W13" s="4">
         <v>250</v>
@@ -781,7 +799,7 @@
         <v>3000</v>
       </c>
       <c r="AC13" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AD13" s="4">
         <v>250</v>
@@ -799,9 +817,9 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:34">
       <c r="A14" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B14" s="4">
         <v>550</v>
@@ -819,7 +837,7 @@
         <v>550</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I14" s="4">
         <v>1100</v>
@@ -837,7 +855,7 @@
         <v>1100</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P14" s="4">
         <v>2200</v>
@@ -855,7 +873,7 @@
         <v>2200</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="W14" s="4">
         <v>3300</v>
@@ -873,7 +891,7 @@
         <v>3300</v>
       </c>
       <c r="AC14" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AD14" s="4">
         <v>4400</v>
@@ -891,9 +909,9 @@
         <v>4400</v>
       </c>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:34">
       <c r="A15" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B15" s="5">
         <f t="shared" ref="B15:D15" si="0">($B$1 - $B$2)/($B$5 + (1 + $B$7)* B13)</f>
@@ -916,7 +934,7 @@
         <v>7.2847682119205301E-6</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="I15" s="5">
         <f>($B$1 - $B$2)/($B$5 + (1 + $B$7)*I13)</f>
@@ -939,7 +957,7 @@
         <v>7.2847682119205301E-6</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="P15" s="5">
         <f>($B$1 - $B$2)/($B$5 + (1 + $B$7)*P13)</f>
@@ -962,7 +980,7 @@
         <v>7.2847682119205301E-6</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="W15" s="5">
         <f>($B$1 - $B$2)/($B$5 + (1 + $B$7)*W13)</f>
@@ -985,7 +1003,7 @@
         <v>7.2847682119205301E-6</v>
       </c>
       <c r="AC15" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="AD15" s="5">
         <f>($B$1 - $B$2)/($B$5 + (1 + $B$7)*AD13)</f>
@@ -1008,9 +1026,9 @@
         <v>7.2847682119205301E-6</v>
       </c>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:34">
       <c r="A16" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B16" s="3">
         <f>$B$7*B15</f>
@@ -1033,7 +1051,7 @@
         <v>2.7682119205298013E-3</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="I16" s="3">
         <f>$B$7 *I15</f>
@@ -1056,7 +1074,7 @@
         <v>2.7682119205298013E-3</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="P16" s="3">
         <f>$B$7 *P15</f>
@@ -1079,7 +1097,7 @@
         <v>2.7682119205298013E-3</v>
       </c>
       <c r="V16" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="W16" s="3">
         <f>$B$7 *W15</f>
@@ -1102,7 +1120,7 @@
         <v>2.7682119205298013E-3</v>
       </c>
       <c r="AC16" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="AD16" s="3">
         <f>$B$7 *AD15</f>
@@ -1125,9 +1143,9 @@
         <v>2.7682119205298013E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:34">
       <c r="A17" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B17" s="3">
         <f>$B$1 - ($B$6 + B13)*B16</f>
@@ -1150,7 +1168,7 @@
         <v>3.927152317880795</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="I17" s="3">
         <f>B1 - ($B$6 + I14)*I16</f>
@@ -1173,7 +1191,7 @@
         <v>-5.8132450331125831</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="P17" s="3">
         <f>I1 - ($B$6 + P14)*P16</f>
@@ -1196,7 +1214,7 @@
         <v>-8.8582781456953636</v>
       </c>
       <c r="V17" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="W17" s="3">
         <f>P1 - ($B$6 + W14)*W16</f>
@@ -1219,7 +1237,7 @@
         <v>-11.903311258278146</v>
       </c>
       <c r="AC17" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="AD17" s="3">
         <f>W1 - ($B$6 + AD14)*AD16</f>
@@ -1242,9 +1260,9 @@
         <v>-14.948344370860926</v>
       </c>
     </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:34">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B18" s="3">
         <f>($B$6*B14)/($B$6+B14)</f>
@@ -1267,7 +1285,7 @@
         <v>354.83870967741933</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I18" s="3">
         <f>($B$6*I14)/($B$6+I14)</f>
@@ -1290,7 +1308,7 @@
         <v>523.80952380952385</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="P18" s="3">
         <f>($B$6*P14)/($B$6+P14)</f>
@@ -1313,7 +1331,7 @@
         <v>687.5</v>
       </c>
       <c r="V18" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="W18" s="3">
         <f>($B$6*W14)/($B$6+W14)</f>
@@ -1336,7 +1354,7 @@
         <v>767.44186046511629</v>
       </c>
       <c r="AC18" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="AD18" s="3">
         <f>($B$6*AD14)/($B$6+AD14)</f>
@@ -1359,9 +1377,9 @@
         <v>814.81481481481478</v>
       </c>
     </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:34">
       <c r="A19" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B19" s="3">
         <f>$B$4/B15</f>
@@ -1384,7 +1402,7 @@
         <v>3431.818181818182</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="I19" s="3">
         <f>$B$4/I15</f>
@@ -1407,7 +1425,7 @@
         <v>3431.818181818182</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="P19" s="3">
         <f>$B$4/P15</f>
@@ -1430,7 +1448,7 @@
         <v>3431.818181818182</v>
       </c>
       <c r="V19" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="W19" s="3">
         <f>$B$4/W15</f>
@@ -1453,7 +1471,7 @@
         <v>3431.818181818182</v>
       </c>
       <c r="AC19" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="AD19" s="3">
         <f>$B$4/AD15</f>
@@ -1476,9 +1494,9 @@
         <v>3431.818181818182</v>
       </c>
     </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:34">
       <c r="A20" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B20" s="3">
         <f>-$B$7*(B18/(B19 + (1 + $B$7)*B13))</f>
@@ -1501,7 +1519,7 @@
         <v>-0.11761598687243921</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="I20" s="3">
         <f>-$B$7*(I18/(I19 + (1+$B$7)*I13))</f>
@@ -1524,7 +1542,7 @@
         <v>-0.17362359966883886</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="P20" s="3">
         <f>-$B$7*(P18/(P19 + (1+$B$7)*P13))</f>
@@ -1547,7 +1565,7 @@
         <v>-0.227880974565351</v>
       </c>
       <c r="V20" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="W20" s="3">
         <f>-$B$7*(W18/(W19 + (1+$B$7)*W13))</f>
@@ -1570,7 +1588,7 @@
         <v>-0.2543787623055081</v>
       </c>
       <c r="AC20" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="AD20" s="3">
         <f>-$B$7*(AD18/(AD19 + (1+$B$7)*AD13))</f>
@@ -1593,9 +1611,9 @@
         <v>-0.27008115504041597</v>
       </c>
     </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:34">
       <c r="A21" s="1" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B21" s="3">
         <f>(B16*(B18 + B13))/SQRT(2)</f>
@@ -1618,7 +1636,7 @@
         <v>6.5668331535444553</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="I21" s="3">
         <f>I16*(I13+I18)</f>
@@ -1641,7 +1659,7 @@
         <v>9.754651529485967</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="P21" s="3">
         <f>P16*(P18+P13)</f>
@@ -1664,7 +1682,7 @@
         <v>10.207781456953642</v>
       </c>
       <c r="V21" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="W21" s="3">
         <f>W16*(W18+W13)</f>
@@ -1687,7 +1705,7 @@
         <v>10.429077468042507</v>
       </c>
       <c r="AC21" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="AD21" s="3">
         <f>AD16*(AD18+AD13)</f>
@@ -1710,9 +1728,9 @@
         <v>10.560215844984057</v>
       </c>
     </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:34">
       <c r="A22" s="7" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="B22" s="8">
         <f>(B18/(B18+B13))*B21</f>
@@ -1735,7 +1753,7 @@
         <v>0.69456889124027887</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="I22" s="8">
         <f>(B18/(B18+B13))*B21</f>
@@ -1758,7 +1776,7 @@
         <v>0.69456889124027887</v>
       </c>
       <c r="O22" s="7" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="P22" s="8">
         <f>(P18/(P18+P13))*P21</f>
@@ -1781,7 +1799,7 @@
         <v>1.9031456953642383</v>
       </c>
       <c r="V22" s="7" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="W22" s="8">
         <f>(W18/(W18+W13))*W21</f>
@@ -1804,7 +1822,7 @@
         <v>2.1244417064531032</v>
       </c>
       <c r="AC22" s="7" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="AD22" s="8">
         <f>(AD18/(AD18+AD13))*AD21</f>
@@ -1827,9 +1845,9 @@
         <v>2.2555800833946531</v>
       </c>
     </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:34">
       <c r="A23" s="1" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B23" s="3">
         <f>ABS(B20)*$B$3</f>
@@ -1852,7 +1870,7 @@
         <v>0.72921911860912314</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="I23" s="3">
         <f>ABS(I20)*$B$3</f>
@@ -1875,7 +1893,7 @@
         <v>1.076466317946801</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="P23" s="3">
         <f>ABS(P20)*$B$3</f>
@@ -1898,7 +1916,7 @@
         <v>1.4128620423051763</v>
       </c>
       <c r="V23" s="1" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="W23" s="3">
         <f>ABS(W20)*$B$3</f>
@@ -1921,7 +1939,7 @@
         <v>1.5771483262941504</v>
       </c>
       <c r="AC23" s="1" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="AD23" s="3">
         <f>ABS(AD20)*$B$3</f>
@@ -1944,9 +1962,9 @@
         <v>1.674503161250579</v>
       </c>
     </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:34">
       <c r="A24" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B24" s="3">
         <f>$B$1*B16</f>
@@ -1969,7 +1987,7 @@
         <v>4.1523178807947023E-2</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="I24" s="3">
         <f>$B$1*I16</f>
@@ -1992,7 +2010,7 @@
         <v>4.1523178807947023E-2</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="P24" s="3">
         <f>$B$1*P16</f>
@@ -2015,7 +2033,7 @@
         <v>4.1523178807947023E-2</v>
       </c>
       <c r="V24" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="W24" s="3">
         <f>$B$1*W16</f>
@@ -2038,7 +2056,7 @@
         <v>4.1523178807947023E-2</v>
       </c>
       <c r="AC24" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="AD24" s="3">
         <f>$B$1*AD16</f>
@@ -2061,9 +2079,9 @@
         <v>4.1523178807947023E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:34">
       <c r="A25" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B25" s="3">
         <f>B37^2/(2*B14)</f>
@@ -2086,7 +2104,7 @@
         <v>4.7746934109554976E-4</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="I25" s="3">
         <f>I37^2/(2*B14)</f>
@@ -2109,7 +2127,7 @@
         <v>8.1605718842031952E-4</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="P25" s="3">
         <f>P37^2/(2*P14)</f>
@@ -2132,7 +2150,7 @@
         <v>4.5367707967880786E-4</v>
       </c>
       <c r="V25" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="W25" s="3">
         <f>W37^2/(W14*2)</f>
@@ -2155,7 +2173,7 @@
         <v>3.7384865155641508E-4</v>
       </c>
       <c r="AC25" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="AD25" s="3">
         <f>AD37^2/(2*AD14)</f>
@@ -2178,126 +2196,126 @@
         <v>3.1863191329979342E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A26" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="3">
+    <row r="26" spans="1:34">
+      <c r="A26" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="10">
         <f>(B25/B24)*100</f>
         <v>28.238345319375131</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C26" s="10">
         <f t="shared" ref="C26:F26" si="64">(C25/C24)*100</f>
         <v>10.27240326809248</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D26" s="10">
         <f t="shared" si="64"/>
         <v>4.2428619440259077</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26" s="10">
         <f t="shared" si="64"/>
         <v>1.8767944677494719</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F26" s="10">
         <f t="shared" si="64"/>
         <v>1.1498862919525998</v>
       </c>
-      <c r="H26" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I26" s="3">
+      <c r="H26" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I26" s="10">
         <f>(I25/I24)*100</f>
         <v>54.656953753645546</v>
       </c>
-      <c r="J26" s="3">
+      <c r="J26" s="10">
         <f t="shared" ref="J26:M26" si="65">(J25/J24)*100</f>
         <v>18.595128528968583</v>
       </c>
-      <c r="K26" s="3">
+      <c r="K26" s="10">
         <f t="shared" si="65"/>
         <v>7.1981384253860039</v>
       </c>
-      <c r="L26" s="3">
+      <c r="L26" s="10">
         <f t="shared" si="65"/>
         <v>3.1125533777514036</v>
       </c>
-      <c r="M26" s="3">
+      <c r="M26" s="10">
         <f t="shared" si="65"/>
         <v>1.9653051906135286</v>
       </c>
-      <c r="O26" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="P26" s="3">
+      <c r="O26" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="P26" s="10">
         <f>(P25/P24)*100</f>
         <v>30.51321999672259</v>
       </c>
-      <c r="Q26" s="3">
+      <c r="Q26" s="10">
         <f>(Q25/Q24)*100</f>
         <v>11.860174627679543</v>
       </c>
-      <c r="R26" s="3">
+      <c r="R26" s="10">
         <f>(R25/R24)*100</f>
         <v>5.0862196103530932</v>
       </c>
-      <c r="S26" s="3">
+      <c r="S26" s="10">
         <f>(S25/S24)*100</f>
         <v>1.9787095277118731</v>
       </c>
-      <c r="T26" s="3">
+      <c r="T26" s="10">
         <f>(T25/T24)*100</f>
         <v>1.0925875443620412</v>
       </c>
-      <c r="V26" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="W26" s="2">
+      <c r="V26" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="W26" s="10">
         <f>(W25/W24)*100</f>
         <v>25.396512450942893</v>
       </c>
-      <c r="X26" s="2">
+      <c r="X26" s="10">
         <f>(X25/X24)*100</f>
         <v>1.0205423561567524</v>
       </c>
-      <c r="Y26" s="2">
+      <c r="Y26" s="10">
         <f>(Y25/Y24)*100</f>
         <v>0.55084312418016756</v>
       </c>
-      <c r="Z26" s="2">
+      <c r="Z26" s="10">
         <f>(Z25/Z24)*100</f>
         <v>0.72559019354956278</v>
       </c>
-      <c r="AA26" s="2">
+      <c r="AA26" s="10">
         <f>(AA25/AA24)*100</f>
         <v>0.9003372629189581</v>
       </c>
-      <c r="AC26" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="AD26" s="3">
+      <c r="AC26" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD26" s="10">
         <f>(AD25/AD24)*100</f>
         <v>21.430409654762649</v>
       </c>
-      <c r="AE26" s="3">
+      <c r="AE26" s="10">
         <f>(AE25/AE24)*100</f>
         <v>8.3297797110725984</v>
       </c>
-      <c r="AF26" s="3">
+      <c r="AF26" s="10">
         <f>(AF25/AF24)*100</f>
         <v>3.5722145960230227</v>
       </c>
-      <c r="AG26" s="3">
+      <c r="AG26" s="10">
         <f>(AG25/AG24)*100</f>
         <v>1.389710944017118</v>
       </c>
-      <c r="AH26" s="3">
+      <c r="AH26" s="10">
         <f>(AH25/AH24)*100</f>
         <v>0.76735915324192672</v>
       </c>
     </row>
-    <row r="35" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:34">
       <c r="A35" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B35" s="6">
         <f>IF(B22&gt;=B23, PI()/2, ASIN(B22/B23))</f>
@@ -2320,7 +2338,7 @@
         <v>1.2612868914214488</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="I35" s="6">
         <f>IF(I22&gt;=I23, PI()/2, ASIN(I22/I23))</f>
@@ -2343,7 +2361,7 @@
         <v>0.70132493979409005</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="P35" s="6">
         <f>IF(P22&gt;=P23, PI()/2, ASIN(P22/P23))</f>
@@ -2366,7 +2384,7 @@
         <v>1.5707963267948966</v>
       </c>
       <c r="V35" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="W35" s="6">
         <f>IF(W21&gt;=W23, PI()/2, ASIN(W21/W23))</f>
@@ -2389,7 +2407,7 @@
         <v>1.5707963267948966</v>
       </c>
       <c r="AC35" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="AD35" s="6">
         <f>IF(AD22&gt;=AD23, PI()/2, ASIN(AD22/AD23))</f>
@@ -2412,9 +2430,9 @@
         <v>1.5707963267948966</v>
       </c>
     </row>
-    <row r="36" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:34">
       <c r="A36" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B36" s="6">
         <f>PI() - B35</f>
@@ -2437,7 +2455,7 @@
         <v>1.8803057621683443</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="I36" s="6">
         <f>PI() - I35</f>
@@ -2460,7 +2478,7 @@
         <v>2.440267713795703</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="P36" s="6">
         <f>PI() - P35</f>
@@ -2483,7 +2501,7 @@
         <v>1.5707963267948966</v>
       </c>
       <c r="V36" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="W36" s="6">
         <f>PI() - W35</f>
@@ -2506,7 +2524,7 @@
         <v>1.5707963267948966</v>
       </c>
       <c r="AC36" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="AD36" s="6">
         <f>PI() - AD35</f>
@@ -2529,7 +2547,7 @@
         <v>1.5707963267948966</v>
       </c>
     </row>
-    <row r="37" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:34">
       <c r="A37" s="1">
         <v>1</v>
       </c>
@@ -2600,7 +2618,7 @@
         <v>1.4128620423051765</v>
       </c>
       <c r="V37" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="W37" s="6">
         <f xml:space="preserve"> (1/PI())*(W23*(PI()/2 + W35 - SIN(2*W35)/2) + 2*W22*COS(W35))</f>
@@ -2623,7 +2641,7 @@
         <v>1.5771483262941504</v>
       </c>
       <c r="AC37" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="AD37" s="6">
         <f xml:space="preserve"> (1/PI())*(AD23*(PI()/2 + AD35 - SIN(2*AD35)/2) + 2*AD22*COS(AD35))</f>
@@ -2646,7 +2664,7 @@
         <v>1.674503161250579</v>
       </c>
     </row>
-    <row r="38" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:34">
       <c r="A38" s="1">
         <v>2</v>
       </c>
@@ -2717,7 +2735,7 @@
         <v>1.9119928209849165E-17</v>
       </c>
       <c r="V38" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="W38" s="6">
         <f>(2/PI()) * ABS( (W23 * COS(W35))/2 - (W23 * COS(3*W35))/6 - (W22 * SIN(2*W35))/2 )</f>
@@ -2740,7 +2758,7 @@
         <v>2.1343175676110696E-17</v>
       </c>
       <c r="AC38" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="AD38" s="6">
         <f>(2/PI()) * ABS( (AD23 * COS(AD35))/2 - (AD23 * COS(3*AD35))/6 - (AD22 * SIN(2*AD35))/2 )</f>
@@ -2763,7 +2781,7 @@
         <v>2.2660655656117555E-17</v>
       </c>
     </row>
-    <row r="39" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:34">
       <c r="A39" s="1">
         <v>3</v>
       </c>
@@ -2834,7 +2852,7 @@
         <v>1.9119928209849149E-17</v>
       </c>
       <c r="V39" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="W39" s="6">
         <f>(2/PI()) * ABS((W23 * SIN(2*W35))/4 - (W23 * SIN(4*W35))/8 + (W22 * COS(3*W35))/3)</f>
@@ -2857,7 +2875,7 @@
         <v>2.1343175676110696E-17</v>
       </c>
       <c r="AC39" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="AD39" s="6">
         <f>(2/PI()) * ABS((AD23 * SIN(2*AD35))/4 - (AD23 * SIN(4*AD35))/8 + (AD22 * COS(3*AD35))/3)</f>
@@ -2880,7 +2898,7 @@
         <v>2.2660655656117555E-17</v>
       </c>
     </row>
-    <row r="40" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:34">
       <c r="A40" s="1">
         <v>4</v>
       </c>
@@ -2951,7 +2969,7 @@
         <v>1.9119928209849174E-17</v>
       </c>
       <c r="V40" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="W40" s="6">
         <f>(2/PI()) * ABS((W23 * COS(3*W35))/6 - (W23 * COS(5*W35))/10 - (W22 * SIN(4*W35))/4)</f>
@@ -2974,7 +2992,7 @@
         <v>2.1343175676110696E-17</v>
       </c>
       <c r="AC40" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="AD40" s="6">
         <f>(2/PI()) * ABS((AD23 * COS(3*AD35))/6 - (AD23 * COS(5*AD35))/10 - (AD22 * SIN(4*AD35))/4)</f>
@@ -2997,7 +3015,7 @@
         <v>2.2660655656117555E-17</v>
       </c>
     </row>
-    <row r="41" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:34">
       <c r="A41" s="1">
         <v>5</v>
       </c>
@@ -3068,7 +3086,7 @@
         <v>1.9119928209849149E-17</v>
       </c>
       <c r="V41" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="W41" s="6">
         <f>(2/PI()) * ABS((W23 * SIN(4*W35))/8 - (W23 * SIN(6*W35))/12 + (W22 * COS(5*W35))/5)</f>
@@ -3091,7 +3109,7 @@
         <v>2.1343175676110696E-17</v>
       </c>
       <c r="AC41" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="AD41" s="6">
         <f>(2/PI()) * ABS((AD23 * SIN(4*AD35))/8 - (AD23 * SIN(6*AD35))/12 + (AD22 * COS(5*AD35))/5)</f>
@@ -3114,7 +3132,7 @@
         <v>2.2660655656117555E-17</v>
       </c>
     </row>
-    <row r="42" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:34">
       <c r="A42" s="1">
         <v>6</v>
       </c>
@@ -3185,7 +3203,7 @@
         <v>1.9119928209849155E-17</v>
       </c>
       <c r="V42" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="W42" s="6">
         <f>(2/PI()) * ABS((W23 * COS(5*W35))/10 - (W23 * COS(7*W35))/14 - (W22 * SIN(6*W35))/6)</f>
@@ -3208,7 +3226,7 @@
         <v>2.1343175676110687E-17</v>
       </c>
       <c r="AC42" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="AD42" s="6">
         <f>(2/PI()) * ABS((AD23 * COS(5*AD35))/10 - (AD23 * COS(7*AD35))/14 - (AD22 * SIN(6*AD35))/6)</f>
@@ -3231,7 +3249,7 @@
         <v>2.2660655656117555E-17</v>
       </c>
     </row>
-    <row r="43" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:34">
       <c r="A43" s="1">
         <v>7</v>
       </c>
@@ -3302,7 +3320,7 @@
         <v>1.9119928209849149E-17</v>
       </c>
       <c r="V43" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="W43" s="6">
         <f>(2/PI()) * ABS((W23 * SIN(6*W35))/12 - (W23 * SIN(8*W35))/16 + (W22 * COS(7*W35))/7)</f>
@@ -3325,7 +3343,7 @@
         <v>2.1343175676110696E-17</v>
       </c>
       <c r="AC43" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="AD43" s="6">
         <f>(2/PI()) * ABS((AD23 * SIN(6*AD35))/12 - (AD23 * SIN(8*AD35))/16 + (AD22 * COS(7*AD35))/7)</f>
@@ -3348,7 +3366,7 @@
         <v>2.2660655656117555E-17</v>
       </c>
     </row>
-    <row r="44" spans="1:34" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:34">
       <c r="A44" s="1">
         <v>8</v>
       </c>
@@ -3419,7 +3437,7 @@
         <v>1.9119928209849174E-17</v>
       </c>
       <c r="V44" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="W44" s="6">
         <f>(2/PI()) * ABS((W23 * COS(7*W35))/14 - (W23 * COS(9*W35))/18 - (W22 * SIN(8*W35))/8)</f>
@@ -3442,7 +3460,7 @@
         <v>2.1343175676110696E-17</v>
       </c>
       <c r="AC44" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="AD44" s="6">
         <f>(2/PI()) * ABS((AD23 * COS(7*AD35))/14 - (AD23 * COS(9*AD35))/18 - (AD22 * SIN(8*AD35))/8)</f>
@@ -3465,119 +3483,119 @@
         <v>2.2660655656117555E-17</v>
       </c>
     </row>
-    <row r="45" spans="1:34" x14ac:dyDescent="0.45">
-      <c r="A45" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B45" s="6">
+    <row r="45" spans="1:34">
+      <c r="A45" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B45" s="10">
         <f>(SQRT(B38^2 + B39^2 + B40^2 + B41^2 + B42^2 + B43^2 + B44^2) / B37)*100</f>
         <v>34.455494252815896</v>
       </c>
-      <c r="C45" s="6">
+      <c r="C45" s="10">
         <f t="shared" ref="C45:F45" si="116">(SQRT(C38^2 + C39^2 + C40^2 + C41^2) / C37)*100</f>
         <v>27.818932987642341</v>
       </c>
-      <c r="D45" s="6">
+      <c r="D45" s="10">
         <f t="shared" si="116"/>
         <v>18.434458663753858</v>
       </c>
-      <c r="E45" s="6">
+      <c r="E45" s="10">
         <f t="shared" si="116"/>
         <v>7.4346607000191263</v>
       </c>
-      <c r="F45" s="6">
+      <c r="F45" s="10">
         <f t="shared" si="116"/>
         <v>1.105188065876713</v>
       </c>
-      <c r="H45" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I45" s="6">
+      <c r="H45" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="I45" s="10">
         <f>(SQRT(I38^2 + I39^2 + I40^2 + I41^2 + I42^2 + I43^2 + I44^2) / I37)*100</f>
         <v>37.258147308652561</v>
       </c>
-      <c r="J45" s="6">
+      <c r="J45" s="10">
         <f t="shared" ref="J45:M45" si="117">(SQRT(J38^2 + J39^2 + J40^2 + J41^2 + J42^2 + J43^2 + J44^2) / J37)*100</f>
         <v>32.613739290927299</v>
       </c>
-      <c r="K45" s="6">
+      <c r="K45" s="10">
         <f t="shared" si="117"/>
         <v>25.962790097978122</v>
       </c>
-      <c r="L45" s="6">
+      <c r="L45" s="10">
         <f t="shared" si="117"/>
         <v>17.962613187663003</v>
       </c>
-      <c r="M45" s="6">
+      <c r="M45" s="10">
         <f t="shared" si="117"/>
         <v>13.302178748613169</v>
       </c>
-      <c r="O45" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="P45" s="6">
+      <c r="O45" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="P45" s="10">
         <f>(SQRT(P38^2 + P39^2 + P40^2 + P41^2 + P42^2 + P43^2 + P44^2) / P37)*100</f>
         <v>30.989711304290914</v>
       </c>
-      <c r="Q45" s="6">
+      <c r="Q45" s="10">
         <f t="shared" ref="Q45:T45" si="118">(SQRT(Q38^2 + Q39^2 + Q40^2 + Q41^2 + Q42^2 + Q43^2 + Q44^2) / Q37)*100</f>
         <v>22.095548003342842</v>
       </c>
-      <c r="R45" s="6">
+      <c r="R45" s="10">
         <f t="shared" si="118"/>
         <v>9.5942972320558901</v>
       </c>
-      <c r="S45" s="6">
+      <c r="S45" s="10">
         <f t="shared" si="118"/>
         <v>1.1863218544948951E-15</v>
       </c>
-      <c r="T45" s="6">
+      <c r="T45" s="10">
         <f t="shared" si="118"/>
         <v>3.5804327396420078E-15</v>
       </c>
-      <c r="V45" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="W45" s="6">
+      <c r="V45" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="W45" s="10">
         <f>(SQRT(W38^2 + W39^2 + W40^2 + W41^2 + W42^2 + W43^2 + W44^2) / W37)*100</f>
         <v>31.348069583918797</v>
       </c>
-      <c r="X45" s="6">
+      <c r="X45" s="10">
         <f t="shared" ref="X45:AA45" si="119">(SQRT(X38^2 + X39^2 + X40^2 + X41^2 + X42^2 + X43^2 + X44^2) / X37)*100</f>
         <v>24.653639811431336</v>
       </c>
-      <c r="Y45" s="6">
+      <c r="Y45" s="10">
         <f t="shared" si="119"/>
         <v>2.726783613901272E-15</v>
       </c>
-      <c r="Z45" s="6">
+      <c r="Z45" s="10">
         <f t="shared" si="119"/>
         <v>1.1863218544948941E-15</v>
       </c>
-      <c r="AA45" s="6">
+      <c r="AA45" s="10">
         <f t="shared" si="119"/>
         <v>3.5804327396420102E-15</v>
       </c>
-      <c r="AC45" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AD45" s="6">
+      <c r="AC45" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD45" s="10">
         <f>(SQRT(AD38^2 + AD39^2 + AD40^2 + AD41^2 + AD42^2 + AD43^2 + AD44^2) / AD37)*100</f>
         <v>30.9897113042909</v>
       </c>
-      <c r="AE45" s="6">
+      <c r="AE45" s="10">
         <f t="shared" ref="AE45:AH45" si="120">(SQRT(AE38^2 + AE39^2 + AE40^2 + AE41^2 + AE42^2 + AE43^2 + AE44^2) / AE37)*100</f>
         <v>22.095548003342845</v>
       </c>
-      <c r="AF45" s="6">
+      <c r="AF45" s="10">
         <f t="shared" si="120"/>
         <v>9.5942972320558884</v>
       </c>
-      <c r="AG45" s="6">
+      <c r="AG45" s="10">
         <f t="shared" si="120"/>
         <v>1.1863218544948945E-15</v>
       </c>
-      <c r="AH45" s="6">
+      <c r="AH45" s="10">
         <f t="shared" si="120"/>
         <v>3.5804327396420149E-15</v>
       </c>
@@ -3598,13 +3616,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB653757-3CF0-4E4B-8DDA-2B5EED0DCAED}">
   <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="11.796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="10.265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3612,7 +3630,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3620,7 +3638,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -3628,15 +3646,15 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -3644,25 +3662,25 @@
         <v>470000</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2">
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2">
         <v>380</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1">
         <v>250</v>
@@ -3680,11 +3698,11 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5">
+        <v>14</v>
+      </c>
+      <c r="B11" s="12">
         <f>($B$1-$B$2)/($B$5+(1+$B$7)*$B6)</f>
         <v>1.6803760282021152E-5</v>
       </c>
@@ -3705,9 +3723,9 @@
         <v>1.6803760282021152E-5</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B12" s="6">
         <f>B11*$B$7</f>
@@ -3730,9 +3748,9 @@
         <v>6.385428907168038E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B13" s="6">
         <f>$B$1-$B$6*B12</f>
@@ -3755,9 +3773,9 @@
         <v>8.6145710928319623</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B14" s="6">
         <f>($B$6*B$10)/($B$6+B$10)</f>
@@ -3780,9 +3798,9 @@
         <v>666.66666666666663</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B15" s="6">
         <f>$B$4/B11</f>
@@ -3805,9 +3823,9 @@
         <v>1487.7622377622379</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B16" s="6">
         <f>((1+$B$7)*B14)/(B15+(1+$B$7)*B14)</f>
@@ -3830,427 +3848,427 @@
         <v>0.99417677690418027</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="6">
+        <v>20</v>
+      </c>
+      <c r="B17" s="3">
         <f>B14*B12</f>
         <v>1.2770857814336076</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="3">
         <f t="shared" ref="C17:F17" si="6">C14*C12</f>
         <v>2.128476302389346</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="3">
         <f t="shared" si="6"/>
         <v>3.1927144535840188</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="3">
         <f t="shared" si="6"/>
         <v>3.8312573443008229</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="3">
         <f t="shared" si="6"/>
         <v>4.2569526047786921</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:6">
       <c r="A18" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="6">
+        <v>22</v>
+      </c>
+      <c r="B18" s="3">
         <f>B14*B12</f>
         <v>1.2770857814336076</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="3">
         <f t="shared" ref="C18:F18" si="7">C14*C12</f>
         <v>2.128476302389346</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="3">
         <f t="shared" si="7"/>
         <v>3.1927144535840188</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="3">
         <f t="shared" si="7"/>
         <v>3.8312573443008229</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="3">
         <f t="shared" si="7"/>
         <v>4.2569526047786921</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" s="6">
+        <v>24</v>
+      </c>
+      <c r="B19" s="3">
         <f>$B$3*B16</f>
         <v>6.0812666807689029</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="3">
         <f t="shared" ref="C19:F19" si="8">$B$3*C16</f>
         <v>6.1282100823185255</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="3">
         <f t="shared" si="8"/>
         <v>6.1519546154056295</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="3">
         <f t="shared" si="8"/>
         <v>6.1599104020812971</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="3">
         <f t="shared" si="8"/>
         <v>6.1638960168059178</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:6">
       <c r="A20" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="6">
+        <v>26</v>
+      </c>
+      <c r="B20" s="3">
         <f>$B$1*B12</f>
         <v>9.5781433607520575E-2</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="3">
         <f t="shared" ref="C20:F20" si="9">$B$1*C12</f>
         <v>9.5781433607520575E-2</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="3">
         <f t="shared" si="9"/>
         <v>9.5781433607520575E-2</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="3">
         <f t="shared" si="9"/>
         <v>9.5781433607520575E-2</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="3">
         <f t="shared" si="9"/>
         <v>9.5781433607520575E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="6">
+        <v>27</v>
+      </c>
+      <c r="B21" s="3">
         <f>B19^2/(2*B10)</f>
         <v>7.396360888526006E-2</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="3">
         <f t="shared" ref="C21:F21" si="10">C19^2/(2*C10)</f>
         <v>3.7554958813030434E-2</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="3">
         <f t="shared" si="10"/>
         <v>1.8923272795005313E-2</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="3">
         <f t="shared" si="10"/>
         <v>1.2648165387223123E-2</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="3">
         <f t="shared" si="10"/>
         <v>9.498403526498965E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="6">
+        <v>28</v>
+      </c>
+      <c r="B22" s="3">
         <f>(B21/B20)*100</f>
         <v>77.221238082881001</v>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="3">
         <f t="shared" ref="C22:F22" si="11">(C21/C20)*100</f>
         <v>39.20901723701251</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="3">
         <f t="shared" si="11"/>
         <v>19.756723283706933</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="3">
         <f t="shared" si="11"/>
         <v>13.205237080759263</v>
       </c>
-      <c r="F22" s="6">
+      <c r="F22" s="3">
         <f t="shared" si="11"/>
         <v>9.9167481303528628</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:6">
       <c r="A26" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="6">
+        <v>29</v>
+      </c>
+      <c r="B26" s="3">
         <f>IF(B17&gt;=B19, PI()/2, ASIN(B17/B19))</f>
         <v>0.21157828629706418</v>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="3">
         <f t="shared" ref="C26:F26" si="12">IF(C17&gt;=C19, PI()/2, ASIN(C17/C19))</f>
         <v>0.35471626074114582</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="3">
         <f t="shared" si="12"/>
         <v>0.54565211180379858</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="3">
         <f t="shared" si="12"/>
         <v>0.67125144173597262</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="3">
         <f t="shared" si="12"/>
         <v>0.76235556912014169</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:6">
       <c r="A27" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="6">
+        <v>30</v>
+      </c>
+      <c r="B27" s="3">
         <f>PI() - B26</f>
         <v>2.930014367292729</v>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="3">
         <f t="shared" ref="C27:F27" si="13">PI() - C26</f>
         <v>2.7868763928486473</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="3">
         <f t="shared" si="13"/>
         <v>2.5959405417859944</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="3">
         <f t="shared" si="13"/>
         <v>2.4703412118538206</v>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="3">
         <f t="shared" si="13"/>
         <v>2.3792370844696515</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:6">
       <c r="A28" s="1">
         <v>1</v>
       </c>
-      <c r="B28" s="6">
+      <c r="B28" s="3">
         <f xml:space="preserve"> (1/PI())*(B19*(PI()/2 + B26 - SIN(2*B26)/2) + 2*B18*COS(B26))</f>
         <v>3.8476353640929055</v>
       </c>
-      <c r="C28" s="6">
+      <c r="C28" s="3">
         <f t="shared" ref="C28:F28" si="14" xml:space="preserve"> (1/PI())*(C19*(PI()/2 + C26 - SIN(2*C26)/2) + 2*C18*COS(C26))</f>
         <v>4.3913757593559266</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="3">
         <f t="shared" si="14"/>
         <v>5.0131871974652622</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="3">
         <f t="shared" si="14"/>
         <v>5.351061710335224</v>
       </c>
-      <c r="F28" s="6">
+      <c r="F28" s="3">
         <f t="shared" si="14"/>
         <v>5.5576847164327043</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:6">
       <c r="A29" s="1">
         <v>2</v>
       </c>
-      <c r="B29" s="6">
+      <c r="B29" s="3">
         <f>(2/PI()) * ABS( (B19 * COS(B26))/2 - (B19 * COS(3*B26))/6 - (B18 * SIN(2*B26))/2 )</f>
         <v>1.2060649005455608</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="3">
         <f t="shared" ref="C29:F29" si="15">(2/PI()) * ABS( (C19 * COS(C26))/2 - (C19 * COS(3*C26))/6 - (C18 * SIN(2*C26))/2 )</f>
         <v>1.0723755179410071</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="3">
         <f t="shared" si="15"/>
         <v>0.81535892617905104</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="3">
         <f t="shared" si="15"/>
         <v>0.62761257472296839</v>
       </c>
-      <c r="F29" s="6">
+      <c r="F29" s="3">
         <f t="shared" si="15"/>
         <v>0.49477711069170843</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:6">
       <c r="A30" s="1">
         <v>3</v>
       </c>
-      <c r="B30" s="6">
+      <c r="B30" s="3">
         <f>(2/PI()) * ABS((B19 * SIN(2*B26))/4 - (B19 * SIN(4*B26))/8 + (B18 * COS(3*B26))/3)</f>
         <v>0.2532775516725288</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="3">
         <f t="shared" ref="C30:F30" si="16">(2/PI()) * ABS((C19 * SIN(2*C26))/4 - (C19 * SIN(4*C26))/8 + (C18 * COS(3*C26))/3)</f>
         <v>0.37246208053239122</v>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="3">
         <f t="shared" si="16"/>
         <v>0.42315140328761347</v>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="3">
         <f t="shared" si="16"/>
         <v>0.39035393850379357</v>
       </c>
-      <c r="F30" s="6">
+      <c r="F30" s="3">
         <f t="shared" si="16"/>
         <v>0.34170639874541248</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:6">
       <c r="A31" s="1">
         <v>4</v>
       </c>
-      <c r="B31" s="6">
+      <c r="B31" s="3">
         <f>(2/PI()) * ABS((B19 * COS(3*B26))/6 - (B19 * COS(5*B26))/10 - (B18 * SIN(4*B26))/4)</f>
         <v>0.17738604858771967</v>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="3">
         <f t="shared" ref="C31:F31" si="17">(2/PI()) * ABS((C19 * COS(3*C26))/6 - (C19 * COS(5*C26))/10 - (C18 * SIN(4*C26))/4)</f>
         <v>5.9236944066380852E-2</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="3">
         <f t="shared" si="17"/>
         <v>0.10045452842344184</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="3">
         <f t="shared" si="17"/>
         <v>0.1658219292727961</v>
       </c>
-      <c r="F31" s="6">
+      <c r="F31" s="3">
         <f t="shared" si="17"/>
         <v>0.18423454866767608</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:6">
       <c r="A32" s="1">
         <v>5</v>
       </c>
-      <c r="B32" s="6">
+      <c r="B32" s="3">
         <f>(2/PI()) * ABS((B19 * SIN(4*B26))/8 - (B19 * SIN(6*B26))/12 + (B18 * COS(5*B26))/5)</f>
         <v>0.13409471339326454</v>
       </c>
-      <c r="C32" s="6">
+      <c r="C32" s="3">
         <f t="shared" ref="C32:F32" si="18">(2/PI()) * ABS((C19 * SIN(4*C26))/8 - (C19 * SIN(6*C26))/12 + (C18 * COS(5*C26))/5)</f>
         <v>0.15158660067946966</v>
       </c>
-      <c r="D32" s="6">
+      <c r="D32" s="3">
         <f t="shared" si="18"/>
         <v>7.1539199691228864E-2</v>
       </c>
-      <c r="E32" s="6">
+      <c r="E32" s="3">
         <f t="shared" si="18"/>
         <v>7.3962467138603957E-3</v>
       </c>
-      <c r="F32" s="6">
+      <c r="F32" s="3">
         <f t="shared" si="18"/>
         <v>5.5747655617472316E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:6">
       <c r="A33" s="1">
         <v>6</v>
       </c>
-      <c r="B33" s="6">
+      <c r="B33" s="3">
         <f>(2/PI()) * ABS((B19 * COS(5*B26))/10 - (B19 * COS(7*B26))/14 - (B18 * SIN(6*B26))/6)</f>
         <v>3.5793555199097341E-2</v>
       </c>
-      <c r="C33" s="6">
+      <c r="C33" s="3">
         <f t="shared" ref="C33:F33" si="19">(2/PI()) * ABS((C19 * COS(5*C26))/10 - (C19 * COS(7*C26))/14 - (C18 * SIN(6*C26))/6)</f>
         <v>4.9826610537369836E-2</v>
       </c>
-      <c r="D33" s="6">
+      <c r="D33" s="3">
         <f t="shared" si="19"/>
         <v>9.609065565407722E-2</v>
       </c>
-      <c r="E33" s="6">
+      <c r="E33" s="3">
         <f t="shared" si="19"/>
         <v>6.4494802547198443E-2</v>
       </c>
-      <c r="F33" s="6">
+      <c r="F33" s="3">
         <f t="shared" si="19"/>
         <v>2.3956474498384329E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:6">
       <c r="A34" s="1">
         <v>7</v>
       </c>
-      <c r="B34" s="6">
+      <c r="B34" s="3">
         <f>(2/PI()) * ABS((B19 * SIN(6*B26))/12 - (B19 * SIN(8*B26))/16 + (B18 * COS(7*B26))/7)</f>
         <v>7.8322501204670741E-2</v>
       </c>
-      <c r="C34" s="6">
+      <c r="C34" s="3">
         <f t="shared" ref="C34:F34" si="20">(2/PI()) * ABS((C19 * SIN(6*C26))/12 - (C19 * SIN(8*C26))/16 + (C18 * COS(7*C26))/7)</f>
         <v>4.9834311091837523E-2</v>
       </c>
-      <c r="D34" s="6">
+      <c r="D34" s="3">
         <f t="shared" si="20"/>
         <v>3.9033461378100806E-2</v>
       </c>
-      <c r="E34" s="6">
+      <c r="E34" s="3">
         <f t="shared" si="20"/>
         <v>6.3868524336633911E-2</v>
       </c>
-      <c r="F34" s="6">
+      <c r="F34" s="3">
         <f t="shared" si="20"/>
         <v>5.2691307590798861E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:6">
       <c r="A35" s="1">
         <v>8</v>
       </c>
-      <c r="B35" s="6">
+      <c r="B35" s="3">
         <f>(2/PI()) * ABS((B19 * COS(7*B26))/14 - (B19 * COS(9*B26))/18 - (B18 * SIN(8*B26))/8)</f>
         <v>5.7004382009424271E-3</v>
       </c>
-      <c r="C35" s="6">
+      <c r="C35" s="3">
         <f t="shared" ref="C35:F35" si="21">(2/PI()) * ABS((C19 * COS(7*C26))/14 - (C19 * COS(9*C26))/18 - (C18 * SIN(8*C26))/8)</f>
         <v>5.4606044065555207E-2</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D35" s="3">
         <f t="shared" si="21"/>
         <v>2.187216349266391E-2</v>
       </c>
-      <c r="E35" s="6">
+      <c r="E35" s="3">
         <f t="shared" si="21"/>
         <v>2.5962562253822329E-2</v>
       </c>
-      <c r="F35" s="6">
+      <c r="F35" s="3">
         <f t="shared" si="21"/>
         <v>4.3297570456780961E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:6">
       <c r="A36" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B36" s="6">
+        <v>39</v>
+      </c>
+      <c r="B36" s="3">
         <f>(SQRT(B29^2 + B30^2 + B31^2 + B32^2 + B33^2 + B34^2 + B35^2) / B28)*100</f>
         <v>32.623775974722847</v>
       </c>
-      <c r="C36" s="6">
+      <c r="C36" s="3">
         <f t="shared" ref="C36:F36" si="22">(SQRT(C29^2 + C30^2 + C31^2 + C32^2 + C33^2 + C34^2 + C35^2) / C28)*100</f>
         <v>26.194154774068945</v>
       </c>
-      <c r="D36" s="6">
+      <c r="D36" s="3">
         <f t="shared" si="22"/>
         <v>18.609019148718925</v>
       </c>
-      <c r="E36" s="6">
+      <c r="E36" s="3">
         <f t="shared" si="22"/>
         <v>14.265821228795605</v>
       </c>
-      <c r="F36" s="6">
+      <c r="F36" s="3">
         <f t="shared" si="22"/>
         <v>11.434370494382486</v>
       </c>
@@ -4259,4 +4277,750 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DB5610C-A527-463E-9998-1E41FD7BBAD0}">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2">
+        <v>100</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="C4" s="2">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="2">
+        <f>(B4-$B$1)^2/($B$3*2)</f>
+        <v>5.000000000000009E-5</v>
+      </c>
+      <c r="C5" s="2">
+        <f t="shared" ref="C5:D5" si="0">(C4-$B$1)^2/($B$3*2)</f>
+        <v>9.2449999999999991E-2</v>
+      </c>
+      <c r="D5" s="2">
+        <f t="shared" si="0"/>
+        <v>1.1704500000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="6">
+        <f>(2/PI())*(((B4-$B$1)*$B$2)/$B$3)</f>
+        <v>9.54929658551373E-3</v>
+      </c>
+      <c r="C6" s="6">
+        <f t="shared" ref="C6:D6" si="1">(2/PI())*(((C4-$B$1)*$B$2)/$B$3)</f>
+        <v>0.41061975317708999</v>
+      </c>
+      <c r="D6" s="6">
+        <f t="shared" si="1"/>
+        <v>1.4610423775835992</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="11">
+        <f>(B5/B6)*100</f>
+        <v>0.52359877559829926</v>
+      </c>
+      <c r="C7" s="11">
+        <f t="shared" ref="C7:D7" si="2">(C5/C6)*100</f>
+        <v>22.51474735072685</v>
+      </c>
+      <c r="D7" s="11">
+        <f t="shared" si="2"/>
+        <v>80.110612666539737</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="3">
+        <f>ASIN($B$1/B4)</f>
+        <v>1.0654358165107389</v>
+      </c>
+      <c r="C11" s="3">
+        <f t="shared" ref="C11:D11" si="3">ASIN($B$1/C4)</f>
+        <v>0.14046141470985579</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" si="3"/>
+        <v>4.3763968740746353E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="8">
+        <f>IF(($B$2+$B$1)/B$4 &gt;= 1, PI()/2, ASIN(($B$2+$B$1)/B$4))</f>
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="C12" s="8">
+        <f t="shared" ref="C12:D12" si="4">IF(($B$2+$B$1)/C$4 &gt;= 1, PI()/2, ASIN(($B$2+$B$1)/C$4))</f>
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="D12" s="8">
+        <f t="shared" si="4"/>
+        <v>1.3768432989955595</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="1">
+        <v>1</v>
+      </c>
+      <c r="B13" s="6">
+        <f>(4/PI()) * ABS( B$4*(B$12/2 - SIN(2*B$12)/4 - B$11/2 + SIN(2*B$11)/4) + $B$1*(COS(B$12) - COS(B$11)) + $B$2*COS(B$12) )</f>
+        <v>4.1636438995008296E-2</v>
+      </c>
+      <c r="C13" s="6">
+        <f t="shared" ref="C13:D13" si="5">(4/PI()) * ABS( C$4*(C$12/2 - SIN(2*C$12)/4 - C$11/2 + SIN(2*C$11)/4) + $B$1*(COS(C$12) - COS(C$11)) + $B$2*COS(C$12) )</f>
+        <v>4.1116524133413455</v>
+      </c>
+      <c r="D13" s="6">
+        <f t="shared" si="5"/>
+        <v>15.059843292556783</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="1">
+        <v>2</v>
+      </c>
+      <c r="B14" s="6">
+        <v>0</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="1">
+        <v>3</v>
+      </c>
+      <c r="B15" s="6">
+        <f>(4/PI()) * ABS( (B$4/2)*( SIN(($A15-1)*B$12)/($A15-1) - SIN(($A15+1)*B$12)/($A15+1) - SIN(($A15-1)*B$11)/($A15-1) + SIN(($A15+1)*B$11)/($A15+1) ) + ($B$1/$A15)*( COS($A15*B$12) - COS($A15*B$11) ) + ($B$2/$A15)*COS($A15*B$12) )</f>
+        <v>3.3709618034614523E-2</v>
+      </c>
+      <c r="C15" s="6">
+        <f t="shared" ref="C15:D15" si="6">(4/PI()) * ABS( (C$4/2)*( SIN(($A15-1)*C$12)/($A15-1) - SIN(($A15+1)*C$12)/($A15+1) - SIN(($A15-1)*C$11)/($A15-1) + SIN(($A15+1)*C$11)/($A15+1) ) + ($B$1/$A15)*( COS($A15*C$12) - COS($A15*C$11) ) + ($B$2/$A15)*COS($A15*C$12) )</f>
+        <v>0.28839774334883073</v>
+      </c>
+      <c r="D15" s="6">
+        <f t="shared" si="6"/>
+        <v>0.24852777091975067</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="1">
+        <v>4</v>
+      </c>
+      <c r="B16" s="6">
+        <v>0</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0</v>
+      </c>
+      <c r="D16" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="1">
+        <v>5</v>
+      </c>
+      <c r="B17" s="6">
+        <f>(4/PI()) * ABS( (B$4/2)*( SIN(($A17-1)*B$12)/($A17-1) - SIN(($A17+1)*B$12)/($A17+1) - SIN(($A17-1)*B$11)/($A17-1) + SIN(($A17+1)*B$11)/($A17+1) ) + ($B$1/$A17)*( COS($A17*B$12) - COS($A17*B$11) ) + ($B$2/$A17)*COS($A15*B$12) )</f>
+        <v>2.1068511271632596E-2</v>
+      </c>
+      <c r="C17" s="6">
+        <f t="shared" ref="C17:D17" si="7">(4/PI()) * ABS( (C$4/2)*( SIN(($A17-1)*C$12)/($A17-1) - SIN(($A17+1)*C$12)/($A17+1) - SIN(($A17-1)*C$11)/($A17-1) + SIN(($A17+1)*C$11)/($A17+1) ) + ($B$1/$A17)*( COS($A17*C$12) - COS($A17*C$11) ) + ($B$2/$A17)*COS($A15*C$12) )</f>
+        <v>0.16399449277787972</v>
+      </c>
+      <c r="D17" s="6">
+        <f t="shared" si="7"/>
+        <v>5.4712655720836763</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1">
+        <v>6</v>
+      </c>
+      <c r="B18" s="6">
+        <v>0</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0</v>
+      </c>
+      <c r="D18" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="1">
+        <v>7</v>
+      </c>
+      <c r="B19" s="6">
+        <f>(4/PI()) * ABS( (B$4/2)*( SIN(($A19-1)*B$12)/($A19-1) - SIN(($A19+1)*B$12)/($A19+1) - SIN(($A19-1)*B$11)/($A19-1) + SIN(($A19+1)*B$11)/($A19+1) ) + ($B$1/$A19)*( COS($A19*B$12) - COS($A19*B$11) ) + ($B$2/$A19)*COS($A19*B$12) )</f>
+        <v>8.4556212648218519E-3</v>
+      </c>
+      <c r="C19" s="6">
+        <f t="shared" ref="C19:D19" si="8">(4/PI()) * ABS( (C$4/2)*( SIN(($A19-1)*C$12)/($A19-1) - SIN(($A19+1)*C$12)/($A19+1) - SIN(($A19-1)*C$11)/($A19-1) + SIN(($A19+1)*C$11)/($A19+1) ) + ($B$1/$A19)*( COS($A19*C$12) - COS($A19*C$11) ) + ($B$2/$A19)*COS($A19*C$12) )</f>
+        <v>0.10782861367197023</v>
+      </c>
+      <c r="D19" s="6">
+        <f t="shared" si="8"/>
+        <v>8.4496864890299617E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="1">
+        <v>8</v>
+      </c>
+      <c r="B20" s="6">
+        <v>0</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0</v>
+      </c>
+      <c r="D20" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="6">
+        <f t="shared" ref="B21:C21" si="9">(SQRT(B15^2 + B17^2 + B19^2) / B13)*100</f>
+        <v>97.610014662874548</v>
+      </c>
+      <c r="C21" s="6">
+        <f t="shared" si="9"/>
+        <v>8.4843585556204175</v>
+      </c>
+      <c r="D21" s="6">
+        <f>(SQRT(D15^2 + D17^2 + D19^2) / D13)*100</f>
+        <v>36.371952256763898</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EACDA74-623B-427D-B0CF-8D8255884647}">
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2">
+        <v>100</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="C4" s="2">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="2">
+        <f>(B4)^2/($B$3*2)</f>
+        <v>3.2000000000000006E-3</v>
+      </c>
+      <c r="C5" s="2">
+        <f>(C4)^2/($B$3*2)</f>
+        <v>0.125</v>
+      </c>
+      <c r="D5" s="2">
+        <f>(D4)^2/($B$3*2)</f>
+        <v>1.28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="6">
+        <f>(2/PI())*(((B4)*$B$2)/$B$3)</f>
+        <v>7.6394372684109757E-2</v>
+      </c>
+      <c r="C6" s="6">
+        <f>(2/PI())*(((C4)*$B$2)/$B$3)</f>
+        <v>0.47746482927568601</v>
+      </c>
+      <c r="D6" s="6">
+        <f>(2/PI())*(((D4)*$B$2)/$B$3)</f>
+        <v>1.5278874536821954</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="11">
+        <f>(B5/B6)*100</f>
+        <v>4.1887902047863923</v>
+      </c>
+      <c r="C7" s="11">
+        <f t="shared" ref="C7:D7" si="0">(C5/C6)*100</f>
+        <v>26.179938779914945</v>
+      </c>
+      <c r="D7" s="11">
+        <f t="shared" si="0"/>
+        <v>83.775804095727807</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="3">
+        <f>ASIN($B$1/B4)</f>
+        <v>1.0654358165107389</v>
+      </c>
+      <c r="C11" s="3">
+        <f t="shared" ref="C11:D11" si="1">ASIN($B$1/C4)</f>
+        <v>0.14046141470985579</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" si="1"/>
+        <v>4.3763968740746353E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="8">
+        <f>IF(($B$2+$B$1)/B$4 &gt;= 1, PI()/2, ASIN(($B$2+$B$1)/B$4))</f>
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="C12" s="8">
+        <f t="shared" ref="C12:D12" si="2">IF(($B$2+$B$1)/C$4 &gt;= 1, PI()/2, ASIN(($B$2+$B$1)/C$4))</f>
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="D12" s="8">
+        <f t="shared" si="2"/>
+        <v>1.3768432989955595</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="1">
+        <v>1</v>
+      </c>
+      <c r="B13" s="6">
+        <f>(4/PI()) * ABS( B$4*(B$12/2 - SIN(2*B$12)/4 - B$11/2 + SIN(2*B$11)/4) + $B$1*(COS(B$12) - COS(B$11)) + $B$2*COS(B$12) )</f>
+        <v>4.1636438995008296E-2</v>
+      </c>
+      <c r="C13" s="6">
+        <f t="shared" ref="C13:D13" si="3">(4/PI()) * ABS( C$4*(C$12/2 - SIN(2*C$12)/4 - C$11/2 + SIN(2*C$11)/4) + $B$1*(COS(C$12) - COS(C$11)) + $B$2*COS(C$12) )</f>
+        <v>4.1116524133413455</v>
+      </c>
+      <c r="D13" s="6">
+        <f t="shared" si="3"/>
+        <v>15.059843292556783</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="1">
+        <v>2</v>
+      </c>
+      <c r="B14" s="6">
+        <v>0</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="1">
+        <v>3</v>
+      </c>
+      <c r="B15" s="6">
+        <f>(4/PI()) * ABS( (B$4/2)*( SIN(($A15-1)*B$12)/($A15-1) - SIN(($A15+1)*B$12)/($A15+1) - SIN(($A15-1)*B$11)/($A15-1) + SIN(($A15+1)*B$11)/($A15+1) ) + ($B$1/$A15)*( COS($A15*B$12) - COS($A15*B$11) ) + ($B$2/$A15)*COS($A15*B$12) )</f>
+        <v>3.3709618034614523E-2</v>
+      </c>
+      <c r="C15" s="6">
+        <f t="shared" ref="C15:D15" si="4">(4/PI()) * ABS( (C$4/2)*( SIN(($A15-1)*C$12)/($A15-1) - SIN(($A15+1)*C$12)/($A15+1) - SIN(($A15-1)*C$11)/($A15-1) + SIN(($A15+1)*C$11)/($A15+1) ) + ($B$1/$A15)*( COS($A15*C$12) - COS($A15*C$11) ) + ($B$2/$A15)*COS($A15*C$12) )</f>
+        <v>0.28839774334883073</v>
+      </c>
+      <c r="D15" s="6">
+        <f t="shared" si="4"/>
+        <v>0.24852777091975067</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="1">
+        <v>4</v>
+      </c>
+      <c r="B16" s="6">
+        <v>0</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0</v>
+      </c>
+      <c r="D16" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="1">
+        <v>5</v>
+      </c>
+      <c r="B17" s="6">
+        <f>(4/PI()) * ABS( (B$4/2)*( SIN(($A17-1)*B$12)/($A17-1) - SIN(($A17+1)*B$12)/($A17+1) - SIN(($A17-1)*B$11)/($A17-1) + SIN(($A17+1)*B$11)/($A17+1) ) + ($B$1/$A17)*( COS($A17*B$12) - COS($A17*B$11) ) + ($B$2/$A17)*COS($A15*B$12) )</f>
+        <v>2.1068511271632596E-2</v>
+      </c>
+      <c r="C17" s="6">
+        <f t="shared" ref="C17:D17" si="5">(4/PI()) * ABS( (C$4/2)*( SIN(($A17-1)*C$12)/($A17-1) - SIN(($A17+1)*C$12)/($A17+1) - SIN(($A17-1)*C$11)/($A17-1) + SIN(($A17+1)*C$11)/($A17+1) ) + ($B$1/$A17)*( COS($A17*C$12) - COS($A17*C$11) ) + ($B$2/$A17)*COS($A15*C$12) )</f>
+        <v>0.16399449277787972</v>
+      </c>
+      <c r="D17" s="6">
+        <f t="shared" si="5"/>
+        <v>5.4712655720836763</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1">
+        <v>6</v>
+      </c>
+      <c r="B18" s="6">
+        <v>0</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0</v>
+      </c>
+      <c r="D18" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="1">
+        <v>7</v>
+      </c>
+      <c r="B19" s="6">
+        <f>(4/PI()) * ABS( (B$4/2)*( SIN(($A19-1)*B$12)/($A19-1) - SIN(($A19+1)*B$12)/($A19+1) - SIN(($A19-1)*B$11)/($A19-1) + SIN(($A19+1)*B$11)/($A19+1) ) + ($B$1/$A19)*( COS($A19*B$12) - COS($A19*B$11) ) + ($B$2/$A19)*COS($A19*B$12) )</f>
+        <v>8.4556212648218519E-3</v>
+      </c>
+      <c r="C19" s="6">
+        <f t="shared" ref="C19:D19" si="6">(4/PI()) * ABS( (C$4/2)*( SIN(($A19-1)*C$12)/($A19-1) - SIN(($A19+1)*C$12)/($A19+1) - SIN(($A19-1)*C$11)/($A19-1) + SIN(($A19+1)*C$11)/($A19+1) ) + ($B$1/$A19)*( COS($A19*C$12) - COS($A19*C$11) ) + ($B$2/$A19)*COS($A19*C$12) )</f>
+        <v>0.10782861367197023</v>
+      </c>
+      <c r="D19" s="6">
+        <f t="shared" si="6"/>
+        <v>8.4496864890299617E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="1">
+        <v>8</v>
+      </c>
+      <c r="B20" s="6">
+        <v>0</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0</v>
+      </c>
+      <c r="D20" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="6">
+        <f t="shared" ref="B21:C21" si="7">(SQRT(B15^2 + B17^2 + B19^2) / B13)*100</f>
+        <v>97.610014662874548</v>
+      </c>
+      <c r="C21" s="6">
+        <f t="shared" si="7"/>
+        <v>8.4843585556204175</v>
+      </c>
+      <c r="D21" s="6">
+        <f>(SQRT(D15^2 + D17^2 + D19^2) / D13)*100</f>
+        <v>36.371952256763898</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="3">
+        <f>ASIN($B$1/B4)</f>
+        <v>1.0654358165107389</v>
+      </c>
+      <c r="C23" s="3">
+        <f t="shared" ref="C23:D23" si="8">ASIN($B$1/C4)</f>
+        <v>0.14046141470985579</v>
+      </c>
+      <c r="D23" s="3">
+        <f t="shared" si="8"/>
+        <v>4.3763968740746353E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="8">
+        <f t="shared" ref="B24:C24" si="9">IF(B4&lt;=$B$2,PI()/2,ASIN($B$2/B4))</f>
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="C24" s="8">
+        <f t="shared" si="9"/>
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="D24" s="8">
+        <f>IF(D4&lt;=$B$2,PI()/2,ASIN($B$2/D4))</f>
+        <v>1.2153751251046732</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="1">
+        <v>1</v>
+      </c>
+      <c r="B25" s="6">
+        <f t="shared" ref="B25:C25" si="10">(4/PI())*ABS(B$4*(B$24/2-SIN(2*B$12)/4)+$B$2*COS(B$12))</f>
+        <v>0.80000000000000115</v>
+      </c>
+      <c r="C25" s="6">
+        <f t="shared" si="10"/>
+        <v>5.0000000000000009</v>
+      </c>
+      <c r="D25" s="6">
+        <f>(4/PI())*ABS(D$4*(D$24/2-SIN(2*D$24)/4)+$B$2*COS(D$24))</f>
+        <v>15.702723943948081</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="1">
+        <v>2</v>
+      </c>
+      <c r="B26" s="6">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="6">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="6">
+        <f>0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="1">
+        <v>3</v>
+      </c>
+      <c r="B27" s="6">
+        <f>(4/PI())*ABS((B$4/2)*(SIN(($A27-1)*B$12)/($A27-1)-SIN(($A27+1)*B$12)/($A27+1))+($B$2/$A27)*(COS($A27*B$12)-COS($A27*PI()/2)))</f>
+        <v>6.2396298438433582E-17</v>
+      </c>
+      <c r="C27" s="6">
+        <f t="shared" ref="C27:D27" si="11">(4/PI())*ABS((C$4/2)*(SIN(($A27-1)*C$12)/($A27-1)-SIN(($A27+1)*C$12)/($A27+1))+($B$2/$A27)*(COS($A27*C$12)-COS($A27*PI()/2)))</f>
+        <v>3.8997686524020987E-16</v>
+      </c>
+      <c r="D27" s="6">
+        <f>(4/PI())*ABS((D$4/2)*(SIN(($A27-1)*D$24)/($A27-1)-SIN(($A27+1)*D$24)/($A27+1))+($B$2/$A27)*(COS($A27*D$24)-COS($A27*PI()/2)))</f>
+        <v>0.2682641975563903</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="1">
+        <v>4</v>
+      </c>
+      <c r="B28" s="6">
+        <v>0</v>
+      </c>
+      <c r="C28" s="6">
+        <v>0</v>
+      </c>
+      <c r="D28" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="1">
+        <v>5</v>
+      </c>
+      <c r="B29" s="6">
+        <f>(4/PI())*ABS((B$4/2)*(SIN(($A29-1)*B$12)/($A29-1)-SIN(($A29+1)*B$12)/($A29+1))+($B$2/$A29)*(COS($A29*B$12)-COS($A29*PI()/2)))</f>
+        <v>6.2396298438433582E-17</v>
+      </c>
+      <c r="C29" s="6">
+        <f t="shared" ref="C29:D29" si="12">(4/PI())*ABS((C$4/2)*(SIN(($A29-1)*C$12)/($A29-1)-SIN(($A29+1)*C$12)/($A29+1))+($B$2/$A29)*(COS($A29*C$12)-COS($A29*PI()/2)))</f>
+        <v>3.8997686524020987E-16</v>
+      </c>
+      <c r="D29" s="6">
+        <f>(4/PI())*ABS((D$4/2)*(SIN(($A29-1)*D$24)/($A29-1)-SIN(($A29+1)*D$24)/($A29+1))+($B$2/$A29)*(COS($A29*D$24)-COS($A29*PI()/2)))</f>
+        <v>0.21628800927983977</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="1">
+        <v>6</v>
+      </c>
+      <c r="B30" s="6">
+        <v>0</v>
+      </c>
+      <c r="C30" s="6">
+        <v>0</v>
+      </c>
+      <c r="D30" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="1">
+        <v>7</v>
+      </c>
+      <c r="B31" s="6">
+        <f>(4/PI())*ABS((B$4/2)*(SIN(($A31-1)*B$12)/($A31-1)-SIN(($A31+1)*B$12)/($A31+1))+($B$2/$A31)*(COS($A31*B$12)-COS($A31*PI()/2)))</f>
+        <v>6.2396298438433582E-17</v>
+      </c>
+      <c r="C31" s="6">
+        <f t="shared" ref="C31:D31" si="13">(4/PI())*ABS((C$4/2)*(SIN(($A31-1)*C$12)/($A31-1)-SIN(($A31+1)*C$12)/($A31+1))+($B$2/$A31)*(COS($A31*C$12)-COS($A31*PI()/2)))</f>
+        <v>3.8997686524020987E-16</v>
+      </c>
+      <c r="D31" s="6">
+        <f>(4/PI())*ABS((D$4/2)*(SIN(($A31-1)*D$24)/($A31-1)-SIN(($A31+1)*D$24)/($A31+1))+($B$2/$A31)*(COS($A31*D$24)-COS($A31*PI()/2)))</f>
+        <v>0.15181085161311419</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="1">
+        <v>8</v>
+      </c>
+      <c r="B32" s="6">
+        <v>0</v>
+      </c>
+      <c r="C32" s="6">
+        <v>0</v>
+      </c>
+      <c r="D32" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="6">
+        <f t="shared" ref="B33:C33" si="14">(SQRT(B27^2 + B29^2 + B31^2) / B25)*100</f>
+        <v>1.3509194887449676E-14</v>
+      </c>
+      <c r="C33" s="6">
+        <f t="shared" si="14"/>
+        <v>1.350919488744969E-14</v>
+      </c>
+      <c r="D33" s="6">
+        <f>(SQRT(D27^2 + D29^2 + D31^2) / D25)*100</f>
+        <v>2.3980153950683083</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>